<commit_message>
se agrega nucleo de calculo (calc), utilidades de control y red de seguridad
</commit_message>
<xml_diff>
--- a/salidas/vigas/Planilla_Vigas_Portico.xlsx
+++ b/salidas/vigas/Planilla_Vigas_Portico.xlsx
@@ -8,14 +8,16 @@
   </bookViews>
   <sheets>
     <sheet name="resultados_Portico 1_vigas" sheetId="1" r:id="rId1"/>
-    <sheet name="resultados_Portico 8_vigas" sheetId="2" r:id="rId2"/>
+    <sheet name="resultados_Portico 2_vigas" sheetId="2" r:id="rId2"/>
+    <sheet name="resultados_Portico 3_vigas" sheetId="3" r:id="rId3"/>
+    <sheet name="resultados_Portico 8_vigas" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="227" uniqueCount="104">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="462" uniqueCount="114">
   <si>
     <t>Piso</t>
   </si>
@@ -263,6 +265,24 @@
     <t>Estribo_2_Peso_kg</t>
   </si>
   <si>
+    <t>Estribo_3_Zona</t>
+  </si>
+  <si>
+    <t>Estribo_3_Diam_mm</t>
+  </si>
+  <si>
+    <t>Estribo_3_Cantidad</t>
+  </si>
+  <si>
+    <t>Estribo_3_Separacion_cm</t>
+  </si>
+  <si>
+    <t>Estribo_3_Longitud_m</t>
+  </si>
+  <si>
+    <t>Estribo_3_Peso_kg</t>
+  </si>
+  <si>
     <t>V0</t>
   </si>
   <si>
@@ -311,16 +331,28 @@
     <t>Auxiliar superior</t>
   </si>
   <si>
+    <t>apoyo_izq</t>
+  </si>
+  <si>
+    <t>empotramiento</t>
+  </si>
+  <si>
     <t>central</t>
   </si>
   <si>
-    <t>empotramiento</t>
+    <t>extremo_libre</t>
   </si>
   <si>
     <t>apoyo_der</t>
   </si>
   <si>
-    <t>extremo_libre</t>
+    <t>V1</t>
+  </si>
+  <si>
+    <t>V1-1.V1-1 T1</t>
+  </si>
+  <si>
+    <t>V1-1.V1-1 tv_izq</t>
   </si>
   <si>
     <t>V0-1.V0-1 T2</t>
@@ -684,10 +716,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:CD3"/>
+  <dimension ref="A1:CJ3"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:82">
+    <row r="1" spans="1:88">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -934,16 +966,34 @@
       <c r="CD1" s="1" t="s">
         <v>81</v>
       </c>
+      <c r="CE1" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="CF1" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="CG1" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="CH1" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="CI1" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="CJ1" s="1" t="s">
+        <v>87</v>
+      </c>
     </row>
-    <row r="2" spans="1:82">
+    <row r="2" spans="1:88">
       <c r="A2" t="s">
-        <v>82</v>
+        <v>88</v>
       </c>
       <c r="B2" t="s">
-        <v>83</v>
+        <v>89</v>
       </c>
       <c r="C2" t="s">
-        <v>85</v>
+        <v>91</v>
       </c>
       <c r="D2">
         <v>4.85</v>
@@ -997,13 +1047,13 @@
         <v>11.61474741659619</v>
       </c>
       <c r="U2" t="s">
-        <v>87</v>
+        <v>93</v>
       </c>
       <c r="V2">
-        <v>19.82966675680652</v>
+        <v>10.93959008033922</v>
       </c>
       <c r="W2">
-        <v>13.47222222222222</v>
+        <v>0.01347222222222222</v>
       </c>
       <c r="X2" t="b">
         <v>0</v>
@@ -1018,7 +1068,7 @@
         <v>118212.9204050461</v>
       </c>
       <c r="AB2" t="s">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="AC2">
         <v>-101.8192009704092</v>
@@ -1051,16 +1101,16 @@
         <v>1</v>
       </c>
       <c r="AM2" t="s">
-        <v>89</v>
+        <v>95</v>
       </c>
       <c r="AN2" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="AO2">
         <v>1</v>
       </c>
       <c r="AP2" t="s">
-        <v>91</v>
+        <v>97</v>
       </c>
       <c r="AQ2">
         <v>10</v>
@@ -1078,7 +1128,7 @@
         <v>2</v>
       </c>
       <c r="AV2" t="s">
-        <v>93</v>
+        <v>99</v>
       </c>
       <c r="AW2">
         <v>16</v>
@@ -1096,7 +1146,7 @@
         <v>3</v>
       </c>
       <c r="BB2" t="s">
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="BC2">
         <v>16</v>
@@ -1114,7 +1164,7 @@
         <v>4</v>
       </c>
       <c r="BH2" t="s">
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="BI2">
         <v>20</v>
@@ -1132,7 +1182,7 @@
         <v>5</v>
       </c>
       <c r="BN2" t="s">
-        <v>97</v>
+        <v>103</v>
       </c>
       <c r="BO2">
         <v>8</v>
@@ -1147,13 +1197,13 @@
         <v>4.0211</v>
       </c>
       <c r="BS2" t="s">
-        <v>98</v>
+        <v>104</v>
       </c>
       <c r="BT2">
         <v>6</v>
       </c>
       <c r="BU2">
-        <v>21</v>
+        <v>8</v>
       </c>
       <c r="BV2">
         <v>16</v>
@@ -1162,36 +1212,54 @@
         <v>1.04</v>
       </c>
       <c r="BX2">
-        <v>4.84848</v>
+        <v>1.84704</v>
       </c>
       <c r="BY2" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="BZ2">
         <v>6</v>
       </c>
       <c r="CA2">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="CB2">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="CC2">
         <v>1.04</v>
       </c>
       <c r="CD2">
+        <v>3.23232</v>
+      </c>
+      <c r="CE2" t="s">
+        <v>108</v>
+      </c>
+      <c r="CF2">
+        <v>6</v>
+      </c>
+      <c r="CG2">
+        <v>13</v>
+      </c>
+      <c r="CH2">
+        <v>12</v>
+      </c>
+      <c r="CI2">
+        <v>1.04</v>
+      </c>
+      <c r="CJ2">
         <v>3.00144</v>
       </c>
     </row>
-    <row r="3" spans="1:82">
+    <row r="3" spans="1:88">
       <c r="A3" t="s">
-        <v>82</v>
+        <v>88</v>
       </c>
       <c r="B3" t="s">
-        <v>84</v>
+        <v>90</v>
       </c>
       <c r="C3" t="s">
-        <v>86</v>
+        <v>92</v>
       </c>
       <c r="D3">
         <v>0.8</v>
@@ -1293,7 +1361,7 @@
         <v>1</v>
       </c>
       <c r="AP3" t="s">
-        <v>92</v>
+        <v>98</v>
       </c>
       <c r="AQ3">
         <v>8</v>
@@ -1311,7 +1379,7 @@
         <v>2</v>
       </c>
       <c r="AV3" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="AW3">
         <v>10</v>
@@ -1326,7 +1394,7 @@
         <v>0.9872000000000001</v>
       </c>
       <c r="BS3" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="BT3">
         <v>6</v>
@@ -1344,7 +1412,7 @@
         <v>0.69264</v>
       </c>
       <c r="BY3" t="s">
-        <v>101</v>
+        <v>107</v>
       </c>
       <c r="BZ3">
         <v>6</v>
@@ -1369,6 +1437,1678 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:CJ5"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:88">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="P1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="R1" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="S1" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="T1" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="U1" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="V1" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="W1" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="X1" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="Y1" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="Z1" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="AA1" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="AB1" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="AC1" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="AD1" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="AE1" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="AF1" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="AG1" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="AH1" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="AI1" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="AJ1" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="AK1" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="AL1" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="AM1" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="AN1" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="AO1" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="AP1" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="AQ1" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="AR1" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="AS1" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="AT1" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="AU1" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="AV1" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="AW1" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="AX1" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="AY1" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="AZ1" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="BA1" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="BB1" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="BC1" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="BD1" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="BE1" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="BF1" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="BG1" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="BH1" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="BI1" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="BJ1" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="BK1" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="BL1" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="BM1" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="BN1" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="BO1" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="BP1" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="BQ1" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="BR1" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="BS1" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="BT1" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="BU1" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="BV1" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="BW1" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="BX1" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="BY1" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="BZ1" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="CA1" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="CB1" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="CC1" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="CD1" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="CE1" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="CF1" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="CG1" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="CH1" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="CI1" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="CJ1" s="1" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="2" spans="1:88">
+      <c r="A2" t="s">
+        <v>88</v>
+      </c>
+      <c r="B2" t="s">
+        <v>89</v>
+      </c>
+      <c r="C2" t="s">
+        <v>91</v>
+      </c>
+      <c r="D2">
+        <v>4.85</v>
+      </c>
+      <c r="E2">
+        <v>20</v>
+      </c>
+      <c r="F2">
+        <v>420</v>
+      </c>
+      <c r="G2">
+        <v>21019.03898849802</v>
+      </c>
+      <c r="H2">
+        <v>20</v>
+      </c>
+      <c r="I2">
+        <v>39</v>
+      </c>
+      <c r="J2">
+        <v>4</v>
+      </c>
+      <c r="K2">
+        <v>0.3782999999999999</v>
+      </c>
+      <c r="L2">
+        <v>907.9199999999998</v>
+      </c>
+      <c r="M2">
+        <v>4.66</v>
+      </c>
+      <c r="N2">
+        <v>4.71238898038469</v>
+      </c>
+      <c r="O2" t="b">
+        <v>1</v>
+      </c>
+      <c r="P2">
+        <v>98865</v>
+      </c>
+      <c r="Q2">
+        <v>78565.53897894402</v>
+      </c>
+      <c r="R2">
+        <v>0.7946749504773583</v>
+      </c>
+      <c r="S2">
+        <v>16.12777068434789</v>
+      </c>
+      <c r="T2">
+        <v>10.51519368814074</v>
+      </c>
+      <c r="U2" t="s">
+        <v>93</v>
+      </c>
+      <c r="V2">
+        <v>10.07658482219961</v>
+      </c>
+      <c r="W2">
+        <v>0.01347222222222222</v>
+      </c>
+      <c r="X2" t="b">
+        <v>0</v>
+      </c>
+      <c r="Y2">
+        <v>40384.85318155408</v>
+      </c>
+      <c r="Z2">
+        <v>109545.1844476849</v>
+      </c>
+      <c r="AA2">
+        <v>123947.265104983</v>
+      </c>
+      <c r="AB2" t="s">
+        <v>94</v>
+      </c>
+      <c r="AC2">
+        <v>-96.0091517193077</v>
+      </c>
+      <c r="AD2">
+        <v>126.6446439025644</v>
+      </c>
+      <c r="AE2">
+        <v>0</v>
+      </c>
+      <c r="AF2" t="b">
+        <v>1</v>
+      </c>
+      <c r="AG2">
+        <v>45</v>
+      </c>
+      <c r="AH2">
+        <v>280</v>
+      </c>
+      <c r="AI2">
+        <v>78.53981633974483</v>
+      </c>
+      <c r="AJ2">
+        <v>0.05864462243427821</v>
+      </c>
+      <c r="AK2">
+        <v>0.1</v>
+      </c>
+      <c r="AL2" t="b">
+        <v>1</v>
+      </c>
+      <c r="AM2" t="s">
+        <v>95</v>
+      </c>
+      <c r="AN2" t="s">
+        <v>96</v>
+      </c>
+      <c r="AO2">
+        <v>1</v>
+      </c>
+      <c r="AP2" t="s">
+        <v>97</v>
+      </c>
+      <c r="AQ2">
+        <v>10</v>
+      </c>
+      <c r="AR2">
+        <v>5</v>
+      </c>
+      <c r="AS2">
+        <v>0.9460000000000001</v>
+      </c>
+      <c r="AT2">
+        <v>2.91841</v>
+      </c>
+      <c r="AU2">
+        <v>2</v>
+      </c>
+      <c r="AV2" t="s">
+        <v>99</v>
+      </c>
+      <c r="AW2">
+        <v>10</v>
+      </c>
+      <c r="AX2">
+        <v>3</v>
+      </c>
+      <c r="AY2">
+        <v>3.33</v>
+      </c>
+      <c r="AZ2">
+        <v>6.16383</v>
+      </c>
+      <c r="BA2">
+        <v>3</v>
+      </c>
+      <c r="BB2" t="s">
+        <v>101</v>
+      </c>
+      <c r="BC2">
+        <v>10</v>
+      </c>
+      <c r="BD2">
+        <v>3</v>
+      </c>
+      <c r="BE2">
+        <v>5.09</v>
+      </c>
+      <c r="BF2">
+        <v>9.42159</v>
+      </c>
+      <c r="BG2">
+        <v>4</v>
+      </c>
+      <c r="BH2" t="s">
+        <v>102</v>
+      </c>
+      <c r="BI2">
+        <v>20</v>
+      </c>
+      <c r="BJ2">
+        <v>4</v>
+      </c>
+      <c r="BK2">
+        <v>2.013999999999999</v>
+      </c>
+      <c r="BL2">
+        <v>19.866096</v>
+      </c>
+      <c r="BM2">
+        <v>5</v>
+      </c>
+      <c r="BN2" t="s">
+        <v>103</v>
+      </c>
+      <c r="BO2">
+        <v>8</v>
+      </c>
+      <c r="BP2">
+        <v>2</v>
+      </c>
+      <c r="BQ2">
+        <v>5.09</v>
+      </c>
+      <c r="BR2">
+        <v>4.0211</v>
+      </c>
+      <c r="BS2" t="s">
+        <v>104</v>
+      </c>
+      <c r="BT2">
+        <v>6</v>
+      </c>
+      <c r="BU2">
+        <v>7</v>
+      </c>
+      <c r="BV2">
+        <v>16</v>
+      </c>
+      <c r="BW2">
+        <v>1.04</v>
+      </c>
+      <c r="BX2">
+        <v>1.61616</v>
+      </c>
+      <c r="BY2" t="s">
+        <v>106</v>
+      </c>
+      <c r="BZ2">
+        <v>6</v>
+      </c>
+      <c r="CA2">
+        <v>14</v>
+      </c>
+      <c r="CB2">
+        <v>16</v>
+      </c>
+      <c r="CC2">
+        <v>1.04</v>
+      </c>
+      <c r="CD2">
+        <v>3.23232</v>
+      </c>
+      <c r="CE2" t="s">
+        <v>108</v>
+      </c>
+      <c r="CF2">
+        <v>6</v>
+      </c>
+      <c r="CG2">
+        <v>14</v>
+      </c>
+      <c r="CH2">
+        <v>12</v>
+      </c>
+      <c r="CI2">
+        <v>1.04</v>
+      </c>
+      <c r="CJ2">
+        <v>3.23232</v>
+      </c>
+    </row>
+    <row r="3" spans="1:88">
+      <c r="A3" t="s">
+        <v>88</v>
+      </c>
+      <c r="B3" t="s">
+        <v>90</v>
+      </c>
+      <c r="C3" t="s">
+        <v>92</v>
+      </c>
+      <c r="D3">
+        <v>0.8</v>
+      </c>
+      <c r="E3">
+        <v>20</v>
+      </c>
+      <c r="F3">
+        <v>420</v>
+      </c>
+      <c r="G3">
+        <v>21019.03898849802</v>
+      </c>
+      <c r="H3">
+        <v>20</v>
+      </c>
+      <c r="I3">
+        <v>39</v>
+      </c>
+      <c r="J3">
+        <v>4</v>
+      </c>
+      <c r="K3">
+        <v>0.0624</v>
+      </c>
+      <c r="L3">
+        <v>149.76</v>
+      </c>
+      <c r="M3">
+        <v>2.87</v>
+      </c>
+      <c r="N3">
+        <v>2.87</v>
+      </c>
+      <c r="O3" t="b">
+        <v>1</v>
+      </c>
+      <c r="P3">
+        <v>0</v>
+      </c>
+      <c r="Q3">
+        <v>0</v>
+      </c>
+      <c r="R3">
+        <v>0</v>
+      </c>
+      <c r="S3">
+        <v>0</v>
+      </c>
+      <c r="T3">
+        <v>0</v>
+      </c>
+      <c r="V3">
+        <v>0.09971727973625456</v>
+      </c>
+      <c r="W3">
+        <v>4.444444444444445</v>
+      </c>
+      <c r="X3" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y3">
+        <v>104966.8190389107</v>
+      </c>
+      <c r="Z3">
+        <v>0</v>
+      </c>
+      <c r="AA3">
+        <v>0</v>
+      </c>
+      <c r="AC3">
+        <v>0</v>
+      </c>
+      <c r="AD3">
+        <v>0</v>
+      </c>
+      <c r="AE3">
+        <v>62.02640054726523</v>
+      </c>
+      <c r="AF3" t="b">
+        <v>1</v>
+      </c>
+      <c r="AG3">
+        <v>0</v>
+      </c>
+      <c r="AH3">
+        <v>0</v>
+      </c>
+      <c r="AI3">
+        <v>0</v>
+      </c>
+      <c r="AJ3">
+        <v>0</v>
+      </c>
+      <c r="AK3">
+        <v>0</v>
+      </c>
+      <c r="AO3">
+        <v>1</v>
+      </c>
+      <c r="AP3" t="s">
+        <v>98</v>
+      </c>
+      <c r="AQ3">
+        <v>8</v>
+      </c>
+      <c r="AR3">
+        <v>6</v>
+      </c>
+      <c r="AS3">
+        <v>1.12</v>
+      </c>
+      <c r="AT3">
+        <v>2.6544</v>
+      </c>
+      <c r="AU3">
+        <v>2</v>
+      </c>
+      <c r="AV3" t="s">
+        <v>100</v>
+      </c>
+      <c r="AW3">
+        <v>10</v>
+      </c>
+      <c r="AX3">
+        <v>2</v>
+      </c>
+      <c r="AY3">
+        <v>0.8</v>
+      </c>
+      <c r="AZ3">
+        <v>0.9872000000000001</v>
+      </c>
+      <c r="BS3" t="s">
+        <v>105</v>
+      </c>
+      <c r="BT3">
+        <v>6</v>
+      </c>
+      <c r="BU3">
+        <v>3</v>
+      </c>
+      <c r="BV3">
+        <v>16</v>
+      </c>
+      <c r="BW3">
+        <v>1.04</v>
+      </c>
+      <c r="BX3">
+        <v>0.69264</v>
+      </c>
+      <c r="BY3" t="s">
+        <v>107</v>
+      </c>
+      <c r="BZ3">
+        <v>6</v>
+      </c>
+      <c r="CA3">
+        <v>3</v>
+      </c>
+      <c r="CB3">
+        <v>16</v>
+      </c>
+      <c r="CC3">
+        <v>1.04</v>
+      </c>
+      <c r="CD3">
+        <v>0.69264</v>
+      </c>
+    </row>
+    <row r="4" spans="1:88">
+      <c r="A4" t="s">
+        <v>109</v>
+      </c>
+      <c r="B4" t="s">
+        <v>110</v>
+      </c>
+      <c r="C4" t="s">
+        <v>91</v>
+      </c>
+      <c r="D4">
+        <v>4.85</v>
+      </c>
+      <c r="E4">
+        <v>20</v>
+      </c>
+      <c r="F4">
+        <v>420</v>
+      </c>
+      <c r="G4">
+        <v>21019.03898849802</v>
+      </c>
+      <c r="H4">
+        <v>20</v>
+      </c>
+      <c r="I4">
+        <v>39</v>
+      </c>
+      <c r="J4">
+        <v>4</v>
+      </c>
+      <c r="K4">
+        <v>0.3782999999999999</v>
+      </c>
+      <c r="L4">
+        <v>907.9199999999998</v>
+      </c>
+      <c r="M4">
+        <v>5.97</v>
+      </c>
+      <c r="N4">
+        <v>6.031857894892403</v>
+      </c>
+      <c r="O4" t="b">
+        <v>1</v>
+      </c>
+      <c r="P4">
+        <v>98865</v>
+      </c>
+      <c r="Q4">
+        <v>79086.29288605761</v>
+      </c>
+      <c r="R4">
+        <v>0.799942273666693</v>
+      </c>
+      <c r="S4">
+        <v>16.66363867253076</v>
+      </c>
+      <c r="T4">
+        <v>11.61474741659619</v>
+      </c>
+      <c r="U4" t="s">
+        <v>93</v>
+      </c>
+      <c r="V4">
+        <v>10.87117733406704</v>
+      </c>
+      <c r="W4">
+        <v>0.01347222222222222</v>
+      </c>
+      <c r="X4" t="b">
+        <v>0</v>
+      </c>
+      <c r="Y4">
+        <v>45820.65641336665</v>
+      </c>
+      <c r="Z4">
+        <v>108790.7640190467</v>
+      </c>
+      <c r="AA4">
+        <v>115913.0946984504</v>
+      </c>
+      <c r="AB4" t="s">
+        <v>94</v>
+      </c>
+      <c r="AC4">
+        <v>-103.1779571372929</v>
+      </c>
+      <c r="AD4">
+        <v>119.4758384845793</v>
+      </c>
+      <c r="AE4">
+        <v>0</v>
+      </c>
+      <c r="AF4" t="b">
+        <v>1</v>
+      </c>
+      <c r="AG4">
+        <v>48</v>
+      </c>
+      <c r="AH4">
+        <v>280</v>
+      </c>
+      <c r="AI4">
+        <v>201.0619298297468</v>
+      </c>
+      <c r="AJ4">
+        <v>0.08196927443267445</v>
+      </c>
+      <c r="AK4">
+        <v>0.1</v>
+      </c>
+      <c r="AL4" t="b">
+        <v>1</v>
+      </c>
+      <c r="AM4" t="s">
+        <v>95</v>
+      </c>
+      <c r="AN4" t="s">
+        <v>96</v>
+      </c>
+      <c r="AO4">
+        <v>1</v>
+      </c>
+      <c r="AP4" t="s">
+        <v>97</v>
+      </c>
+      <c r="AQ4">
+        <v>16</v>
+      </c>
+      <c r="AR4">
+        <v>2</v>
+      </c>
+      <c r="AS4">
+        <v>1.162</v>
+      </c>
+      <c r="AT4">
+        <v>3.667272</v>
+      </c>
+      <c r="AU4">
+        <v>2</v>
+      </c>
+      <c r="AV4" t="s">
+        <v>99</v>
+      </c>
+      <c r="AW4">
+        <v>16</v>
+      </c>
+      <c r="AX4">
+        <v>1</v>
+      </c>
+      <c r="AY4">
+        <v>3.835</v>
+      </c>
+      <c r="AZ4">
+        <v>6.051629999999999</v>
+      </c>
+      <c r="BA4">
+        <v>3</v>
+      </c>
+      <c r="BB4" t="s">
+        <v>101</v>
+      </c>
+      <c r="BC4">
+        <v>16</v>
+      </c>
+      <c r="BD4">
+        <v>2</v>
+      </c>
+      <c r="BE4">
+        <v>5.234</v>
+      </c>
+      <c r="BF4">
+        <v>16.518504</v>
+      </c>
+      <c r="BG4">
+        <v>4</v>
+      </c>
+      <c r="BH4" t="s">
+        <v>102</v>
+      </c>
+      <c r="BI4">
+        <v>16</v>
+      </c>
+      <c r="BJ4">
+        <v>4</v>
+      </c>
+      <c r="BK4">
+        <v>1.517</v>
+      </c>
+      <c r="BL4">
+        <v>9.575303999999999</v>
+      </c>
+      <c r="BM4">
+        <v>5</v>
+      </c>
+      <c r="BN4" t="s">
+        <v>103</v>
+      </c>
+      <c r="BO4">
+        <v>8</v>
+      </c>
+      <c r="BP4">
+        <v>2</v>
+      </c>
+      <c r="BQ4">
+        <v>5.09</v>
+      </c>
+      <c r="BR4">
+        <v>4.0211</v>
+      </c>
+      <c r="BS4" t="s">
+        <v>104</v>
+      </c>
+      <c r="BT4">
+        <v>6</v>
+      </c>
+      <c r="BU4">
+        <v>8</v>
+      </c>
+      <c r="BV4">
+        <v>16</v>
+      </c>
+      <c r="BW4">
+        <v>1.04</v>
+      </c>
+      <c r="BX4">
+        <v>1.84704</v>
+      </c>
+      <c r="BY4" t="s">
+        <v>106</v>
+      </c>
+      <c r="BZ4">
+        <v>6</v>
+      </c>
+      <c r="CA4">
+        <v>14</v>
+      </c>
+      <c r="CB4">
+        <v>16</v>
+      </c>
+      <c r="CC4">
+        <v>1.04</v>
+      </c>
+      <c r="CD4">
+        <v>3.23232</v>
+      </c>
+      <c r="CE4" t="s">
+        <v>108</v>
+      </c>
+      <c r="CF4">
+        <v>6</v>
+      </c>
+      <c r="CG4">
+        <v>13</v>
+      </c>
+      <c r="CH4">
+        <v>12</v>
+      </c>
+      <c r="CI4">
+        <v>1.04</v>
+      </c>
+      <c r="CJ4">
+        <v>3.00144</v>
+      </c>
+    </row>
+    <row r="5" spans="1:88">
+      <c r="A5" t="s">
+        <v>109</v>
+      </c>
+      <c r="B5" t="s">
+        <v>111</v>
+      </c>
+      <c r="C5" t="s">
+        <v>92</v>
+      </c>
+      <c r="D5">
+        <v>0.8</v>
+      </c>
+      <c r="E5">
+        <v>20</v>
+      </c>
+      <c r="F5">
+        <v>420</v>
+      </c>
+      <c r="G5">
+        <v>21019.03898849802</v>
+      </c>
+      <c r="H5">
+        <v>20</v>
+      </c>
+      <c r="I5">
+        <v>39</v>
+      </c>
+      <c r="J5">
+        <v>4</v>
+      </c>
+      <c r="K5">
+        <v>0.0624</v>
+      </c>
+      <c r="L5">
+        <v>149.76</v>
+      </c>
+      <c r="M5">
+        <v>1.17</v>
+      </c>
+      <c r="N5">
+        <v>2.27</v>
+      </c>
+      <c r="O5" t="b">
+        <v>1</v>
+      </c>
+      <c r="P5">
+        <v>0</v>
+      </c>
+      <c r="Q5">
+        <v>0</v>
+      </c>
+      <c r="R5">
+        <v>0</v>
+      </c>
+      <c r="S5">
+        <v>0</v>
+      </c>
+      <c r="T5">
+        <v>0</v>
+      </c>
+      <c r="V5">
+        <v>0.1009638843406386</v>
+      </c>
+      <c r="W5">
+        <v>4.444444444444445</v>
+      </c>
+      <c r="X5" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y5">
+        <v>103670.7900600733</v>
+      </c>
+      <c r="Z5">
+        <v>0</v>
+      </c>
+      <c r="AA5">
+        <v>0</v>
+      </c>
+      <c r="AC5">
+        <v>0</v>
+      </c>
+      <c r="AD5">
+        <v>0</v>
+      </c>
+      <c r="AE5">
+        <v>36.72640054726908</v>
+      </c>
+      <c r="AF5" t="b">
+        <v>1</v>
+      </c>
+      <c r="AG5">
+        <v>0</v>
+      </c>
+      <c r="AH5">
+        <v>0</v>
+      </c>
+      <c r="AI5">
+        <v>0</v>
+      </c>
+      <c r="AJ5">
+        <v>0</v>
+      </c>
+      <c r="AK5">
+        <v>0</v>
+      </c>
+      <c r="AO5">
+        <v>1</v>
+      </c>
+      <c r="AP5" t="s">
+        <v>98</v>
+      </c>
+      <c r="AQ5">
+        <v>10</v>
+      </c>
+      <c r="AR5">
+        <v>3</v>
+      </c>
+      <c r="AS5">
+        <v>1.2</v>
+      </c>
+      <c r="AT5">
+        <v>2.221200000000001</v>
+      </c>
+      <c r="AU5">
+        <v>2</v>
+      </c>
+      <c r="AV5" t="s">
+        <v>100</v>
+      </c>
+      <c r="AW5">
+        <v>10</v>
+      </c>
+      <c r="AX5">
+        <v>2</v>
+      </c>
+      <c r="AY5">
+        <v>0.8</v>
+      </c>
+      <c r="AZ5">
+        <v>0.9872000000000001</v>
+      </c>
+      <c r="BS5" t="s">
+        <v>105</v>
+      </c>
+      <c r="BT5">
+        <v>6</v>
+      </c>
+      <c r="BU5">
+        <v>3</v>
+      </c>
+      <c r="BV5">
+        <v>16</v>
+      </c>
+      <c r="BW5">
+        <v>1.04</v>
+      </c>
+      <c r="BX5">
+        <v>0.69264</v>
+      </c>
+      <c r="BY5" t="s">
+        <v>107</v>
+      </c>
+      <c r="BZ5">
+        <v>6</v>
+      </c>
+      <c r="CA5">
+        <v>3</v>
+      </c>
+      <c r="CB5">
+        <v>16</v>
+      </c>
+      <c r="CC5">
+        <v>1.04</v>
+      </c>
+      <c r="CD5">
+        <v>0.69264</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:CD2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:82">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="P1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="R1" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="S1" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="T1" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="U1" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="V1" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="W1" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="X1" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="Y1" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="Z1" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="AA1" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="AB1" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="AC1" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="AD1" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="AE1" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="AF1" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="AG1" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="AH1" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="AI1" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="AJ1" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="AK1" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="AL1" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="AM1" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="AN1" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="AO1" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="AP1" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="AQ1" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="AR1" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="AS1" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="AT1" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="AU1" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="AV1" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="AW1" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="AX1" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="AY1" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="AZ1" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="BA1" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="BB1" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="BC1" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="BD1" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="BE1" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="BF1" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="BG1" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="BH1" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="BI1" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="BJ1" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="BK1" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="BL1" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="BM1" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="BN1" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="BO1" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="BP1" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="BQ1" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="BR1" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="BS1" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="BT1" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="BU1" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="BV1" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="BW1" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="BX1" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="BY1" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="BZ1" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="CA1" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="CB1" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="CC1" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="CD1" s="1" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="2" spans="1:82">
+      <c r="A2" t="s">
+        <v>88</v>
+      </c>
+      <c r="B2" t="s">
+        <v>89</v>
+      </c>
+      <c r="C2" t="s">
+        <v>91</v>
+      </c>
+      <c r="D2">
+        <v>4.2</v>
+      </c>
+      <c r="E2">
+        <v>20</v>
+      </c>
+      <c r="F2">
+        <v>420</v>
+      </c>
+      <c r="G2">
+        <v>21019.03898849802</v>
+      </c>
+      <c r="H2">
+        <v>20</v>
+      </c>
+      <c r="I2">
+        <v>34</v>
+      </c>
+      <c r="J2">
+        <v>4</v>
+      </c>
+      <c r="K2">
+        <v>0.2856</v>
+      </c>
+      <c r="L2">
+        <v>685.4400000000001</v>
+      </c>
+      <c r="M2">
+        <v>1.98</v>
+      </c>
+      <c r="N2">
+        <v>2.010619298297468</v>
+      </c>
+      <c r="O2" t="b">
+        <v>1</v>
+      </c>
+      <c r="P2">
+        <v>65506.66666666668</v>
+      </c>
+      <c r="Q2">
+        <v>53606.18711452316</v>
+      </c>
+      <c r="R2">
+        <v>0.818331779684355</v>
+      </c>
+      <c r="S2">
+        <v>11.44162739098395</v>
+      </c>
+      <c r="T2">
+        <v>6.693909985911229</v>
+      </c>
+      <c r="U2" t="s">
+        <v>93</v>
+      </c>
+      <c r="V2">
+        <v>1.458635083005919</v>
+      </c>
+      <c r="W2">
+        <v>0.01166666666666667</v>
+      </c>
+      <c r="X2" t="b">
+        <v>0</v>
+      </c>
+      <c r="Y2">
+        <v>36316.99754366067</v>
+      </c>
+      <c r="Z2">
+        <v>69663.26574525471</v>
+      </c>
+      <c r="AA2">
+        <v>72127.48762551659</v>
+      </c>
+      <c r="AB2" t="s">
+        <v>94</v>
+      </c>
+      <c r="AC2">
+        <v>-21.22316128604817</v>
+      </c>
+      <c r="AD2">
+        <v>40.6176359055716</v>
+      </c>
+      <c r="AE2">
+        <v>0</v>
+      </c>
+      <c r="AF2" t="b">
+        <v>1</v>
+      </c>
+      <c r="AG2">
+        <v>44</v>
+      </c>
+      <c r="AH2">
+        <v>280</v>
+      </c>
+      <c r="AI2">
+        <v>50.2654824574367</v>
+      </c>
+      <c r="AJ2">
+        <v>0.05016123726069088</v>
+      </c>
+      <c r="AK2">
+        <v>0.1</v>
+      </c>
+      <c r="AL2" t="b">
+        <v>1</v>
+      </c>
+      <c r="AM2" t="s">
+        <v>95</v>
+      </c>
+      <c r="AN2" t="s">
+        <v>96</v>
+      </c>
+      <c r="AO2">
+        <v>1</v>
+      </c>
+      <c r="AP2" t="s">
+        <v>97</v>
+      </c>
+      <c r="AQ2">
+        <v>8</v>
+      </c>
+      <c r="AR2">
+        <v>4</v>
+      </c>
+      <c r="AS2">
+        <v>0.95</v>
+      </c>
+      <c r="AT2">
+        <v>1.501</v>
+      </c>
+      <c r="AU2">
+        <v>2</v>
+      </c>
+      <c r="AV2" t="s">
+        <v>99</v>
+      </c>
+      <c r="AW2">
+        <v>8</v>
+      </c>
+      <c r="AX2">
+        <v>2</v>
+      </c>
+      <c r="AY2">
+        <v>3.132</v>
+      </c>
+      <c r="AZ2">
+        <v>2.47428</v>
+      </c>
+      <c r="BA2">
+        <v>3</v>
+      </c>
+      <c r="BB2" t="s">
+        <v>101</v>
+      </c>
+      <c r="BC2">
+        <v>8</v>
+      </c>
+      <c r="BD2">
+        <v>2</v>
+      </c>
+      <c r="BE2">
+        <v>4.392</v>
+      </c>
+      <c r="BF2">
+        <v>3.46968</v>
+      </c>
+      <c r="BG2">
+        <v>4</v>
+      </c>
+      <c r="BH2" t="s">
+        <v>102</v>
+      </c>
+      <c r="BI2">
+        <v>10</v>
+      </c>
+      <c r="BJ2">
+        <v>5</v>
+      </c>
+      <c r="BK2">
+        <v>1.03</v>
+      </c>
+      <c r="BL2">
+        <v>3.177550000000001</v>
+      </c>
+      <c r="BM2">
+        <v>5</v>
+      </c>
+      <c r="BN2" t="s">
+        <v>103</v>
+      </c>
+      <c r="BO2">
+        <v>8</v>
+      </c>
+      <c r="BP2">
+        <v>2</v>
+      </c>
+      <c r="BQ2">
+        <v>4.44</v>
+      </c>
+      <c r="BR2">
+        <v>3.5076</v>
+      </c>
+      <c r="BS2" t="s">
+        <v>106</v>
+      </c>
+      <c r="BT2">
+        <v>6</v>
+      </c>
+      <c r="BU2">
+        <v>28</v>
+      </c>
+      <c r="BV2">
+        <v>14</v>
+      </c>
+      <c r="BW2">
+        <v>0.9400000000000001</v>
+      </c>
+      <c r="BX2">
+        <v>5.84304</v>
+      </c>
+      <c r="BY2" t="s">
+        <v>108</v>
+      </c>
+      <c r="BZ2">
+        <v>6</v>
+      </c>
+      <c r="CA2">
+        <v>3</v>
+      </c>
+      <c r="CB2">
+        <v>14</v>
+      </c>
+      <c r="CC2">
+        <v>0.9400000000000001</v>
+      </c>
+      <c r="CD2">
+        <v>0.62604</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:CD5"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
@@ -1622,13 +3362,13 @@
     </row>
     <row r="2" spans="1:82">
       <c r="A2" t="s">
-        <v>82</v>
+        <v>88</v>
       </c>
       <c r="B2" t="s">
-        <v>83</v>
+        <v>89</v>
       </c>
       <c r="C2" t="s">
-        <v>85</v>
+        <v>91</v>
       </c>
       <c r="D2">
         <v>4</v>
@@ -1682,7 +3422,7 @@
         <v>9.328569808260646</v>
       </c>
       <c r="U2" t="s">
-        <v>87</v>
+        <v>93</v>
       </c>
       <c r="V2">
         <v>9.543068675366721</v>
@@ -1703,7 +3443,7 @@
         <v>124957.9010004124</v>
       </c>
       <c r="AB2" t="s">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="AC2">
         <v>-83.994257678049</v>
@@ -1736,16 +3476,16 @@
         <v>1</v>
       </c>
       <c r="AM2" t="s">
-        <v>89</v>
+        <v>95</v>
       </c>
       <c r="AN2" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="AO2">
         <v>1</v>
       </c>
       <c r="AP2" t="s">
-        <v>91</v>
+        <v>97</v>
       </c>
       <c r="AQ2">
         <v>8</v>
@@ -1763,7 +3503,7 @@
         <v>2</v>
       </c>
       <c r="AV2" t="s">
-        <v>93</v>
+        <v>99</v>
       </c>
       <c r="AW2">
         <v>12</v>
@@ -1781,7 +3521,7 @@
         <v>3</v>
       </c>
       <c r="BB2" t="s">
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="BC2">
         <v>12</v>
@@ -1799,7 +3539,7 @@
         <v>4</v>
       </c>
       <c r="BH2" t="s">
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="BI2">
         <v>16</v>
@@ -1817,7 +3557,7 @@
         <v>5</v>
       </c>
       <c r="BN2" t="s">
-        <v>97</v>
+        <v>103</v>
       </c>
       <c r="BO2">
         <v>8</v>
@@ -1832,7 +3572,7 @@
         <v>3.3496</v>
       </c>
       <c r="BS2" t="s">
-        <v>98</v>
+        <v>106</v>
       </c>
       <c r="BT2">
         <v>6</v>
@@ -1850,7 +3590,7 @@
         <v>3.76512</v>
       </c>
       <c r="BY2" t="s">
-        <v>100</v>
+        <v>108</v>
       </c>
       <c r="BZ2">
         <v>6</v>
@@ -1870,13 +3610,13 @@
     </row>
     <row r="3" spans="1:82">
       <c r="A3" t="s">
-        <v>82</v>
+        <v>88</v>
       </c>
       <c r="B3" t="s">
-        <v>102</v>
+        <v>112</v>
       </c>
       <c r="C3" t="s">
-        <v>85</v>
+        <v>91</v>
       </c>
       <c r="D3">
         <v>5</v>
@@ -1930,7 +3670,7 @@
         <v>10.51899050410677</v>
       </c>
       <c r="U3" t="s">
-        <v>87</v>
+        <v>93</v>
       </c>
       <c r="V3">
         <v>23.38295401739195</v>
@@ -1951,7 +3691,7 @@
         <v>127432.6800952257</v>
       </c>
       <c r="AB3" t="s">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="AC3">
         <v>-102.7880992746242</v>
@@ -1984,16 +3724,16 @@
         <v>1</v>
       </c>
       <c r="AM3" t="s">
-        <v>89</v>
+        <v>95</v>
       </c>
       <c r="AN3" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="AO3">
         <v>1</v>
       </c>
       <c r="AP3" t="s">
-        <v>91</v>
+        <v>97</v>
       </c>
       <c r="AQ3">
         <v>12</v>
@@ -2011,7 +3751,7 @@
         <v>2</v>
       </c>
       <c r="AV3" t="s">
-        <v>93</v>
+        <v>99</v>
       </c>
       <c r="AW3">
         <v>12</v>
@@ -2029,7 +3769,7 @@
         <v>3</v>
       </c>
       <c r="BB3" t="s">
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="BC3">
         <v>12</v>
@@ -2047,7 +3787,7 @@
         <v>4</v>
       </c>
       <c r="BH3" t="s">
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="BI3">
         <v>20</v>
@@ -2065,7 +3805,7 @@
         <v>5</v>
       </c>
       <c r="BN3" t="s">
-        <v>97</v>
+        <v>103</v>
       </c>
       <c r="BO3">
         <v>8</v>
@@ -2080,7 +3820,7 @@
         <v>4.139600000000001</v>
       </c>
       <c r="BS3" t="s">
-        <v>98</v>
+        <v>106</v>
       </c>
       <c r="BT3">
         <v>6</v>
@@ -2098,7 +3838,7 @@
         <v>4.94172</v>
       </c>
       <c r="BY3" t="s">
-        <v>100</v>
+        <v>108</v>
       </c>
       <c r="BZ3">
         <v>6</v>
@@ -2118,13 +3858,13 @@
     </row>
     <row r="4" spans="1:82">
       <c r="A4" t="s">
-        <v>82</v>
+        <v>88</v>
       </c>
       <c r="B4" t="s">
-        <v>84</v>
+        <v>90</v>
       </c>
       <c r="C4" t="s">
-        <v>86</v>
+        <v>92</v>
       </c>
       <c r="D4">
         <v>1.2</v>
@@ -2226,7 +3966,7 @@
         <v>1</v>
       </c>
       <c r="AP4" t="s">
-        <v>92</v>
+        <v>98</v>
       </c>
       <c r="AQ4">
         <v>10</v>
@@ -2244,7 +3984,7 @@
         <v>2</v>
       </c>
       <c r="AV4" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="AW4">
         <v>10</v>
@@ -2259,7 +3999,7 @@
         <v>1.4808</v>
       </c>
       <c r="BS4" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="BT4">
         <v>6</v>
@@ -2277,7 +4017,7 @@
         <v>0.94128</v>
       </c>
       <c r="BY4" t="s">
-        <v>101</v>
+        <v>107</v>
       </c>
       <c r="BZ4">
         <v>6</v>
@@ -2297,13 +4037,13 @@
     </row>
     <row r="5" spans="1:82">
       <c r="A5" t="s">
-        <v>82</v>
+        <v>88</v>
       </c>
       <c r="B5" t="s">
-        <v>103</v>
+        <v>113</v>
       </c>
       <c r="C5" t="s">
-        <v>86</v>
+        <v>92</v>
       </c>
       <c r="D5">
         <v>1.3</v>
@@ -2405,7 +4145,7 @@
         <v>1</v>
       </c>
       <c r="AP5" t="s">
-        <v>92</v>
+        <v>98</v>
       </c>
       <c r="AQ5">
         <v>8</v>
@@ -2423,7 +4163,7 @@
         <v>2</v>
       </c>
       <c r="AV5" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="AW5">
         <v>10</v>
@@ -2438,7 +4178,7 @@
         <v>1.6042</v>
       </c>
       <c r="BS5" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="BT5">
         <v>6</v>
@@ -2456,7 +4196,7 @@
         <v>0.70596</v>
       </c>
       <c r="BY5" t="s">
-        <v>101</v>
+        <v>107</v>
       </c>
       <c r="BZ5">
         <v>6</v>

</xml_diff>